<commit_message>
scan: seg5 2026-10-26 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq6_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>78.90131148220883</v>
+        <v>78.90131156175438</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>33.15849057183254</v>
+        <v>33.15849061754602</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.887832827195892</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.1917634644417778</v>
+        <v>0.1917634640524146</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>88.80743659518778</v>
+        <v>88.80743663051797</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>40.42124230723691</v>
+        <v>40.42124236999416</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>4.685271930498494</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2.338155083939738</v>
+        <v>2.338155083809959</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>67.03613213401631</v>
+        <v>67.03613243533684</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>19.45238165251561</v>
+        <v>19.45238169571356</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.026592574560778</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.04737782222289627</v>
+        <v>0.04737782209310933</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65.64072220204432</v>
+        <v>65.6407222068942</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>34.890155062347</v>
+        <v>34.89015513951923</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.416036974209795</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-0.3201726229756376</v>
+        <v>-0.3201726229496833</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55.08568304782916</v>
+        <v>55.0856830495019</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>36.65148666452099</v>
+        <v>36.65148684351382</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.233027650764054</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-5.186169113455673</v>
+        <v>-5.186169113878286</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>857.237312605263</v>
+        <v>857.2373126052629</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>90.09999999999999</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.41895108188609</v>
+        <v>60.41895069619824</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>33.02733244354248</v>
+        <v>33.02733246566626</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.281559472437751</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.02741526892322721</v>
+        <v>0.02741526840408426</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>54.64295262449493</v>
+        <v>54.64295263835304</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>33.47085422785257</v>
+        <v>33.47085421456798</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.6145525805647692</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-0.6052151002842892</v>
+        <v>-0.6052151005438731</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>66.14815018164282</v>
+        <v>66.14815023444106</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>33.13629603199323</v>
+        <v>33.13629602100019</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2.544511166061138</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.7480122025300724</v>
+        <v>0.7480122021666666</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>60.06618486530025</v>
+        <v>60.06618490310662</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>49.94953713038884</v>
+        <v>49.94953734204721</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.398229788631511</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.547504951229226</v>
+        <v>1.547504950749008</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>59.64192345871853</v>
+        <v>59.64192344313563</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>26.41004630783667</v>
+        <v>26.41004659100323</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>3.166044129630837</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>2.003902512995683</v>
+        <v>2.003902512580358</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>712.1949567710934</v>
+        <v>712.1949567710933</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>26.85</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>82.00485215658971</v>
+        <v>82.00485241673489</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>52.30388539492535</v>
+        <v>52.30388558433571</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.033008627467827</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.2300014572477103</v>
+        <v>0.2300014569881352</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>49.94045097420253</v>
+        <v>49.94045106699661</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>36.37853756754624</v>
+        <v>36.37853757561509</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.6998040680600051</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-0.9585343456074904</v>
+        <v>-0.9585343487223748</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>677.0219967973202</v>
+        <v>677.0219967973212</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>45.9</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>68.14931605877572</v>
+        <v>68.14931598112399</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>35.44148197183497</v>
+        <v>35.44148194933189</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.6476559223050367</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.2317171874937166</v>
+        <v>0.2317171873639329</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>69.44974521961467</v>
+        <v>69.44974491603531</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>41.35617004318013</v>
+        <v>41.35617015557782</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>5.971524141804417</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.07751029843398038</v>
+        <v>0.07751029840802381</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>64.81172466953879</v>
+        <v>64.81172467745395</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>51.30590219839804</v>
+        <v>51.3059022253042</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.252859594182261</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3.795119548270154</v>
+        <v>3.795119547750986</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>53.90440080384538</v>
+        <v>53.90440152316441</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>28.80512445100012</v>
+        <v>28.80512429673319</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.6183082921517314</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.102891322796602</v>
+        <v>0.1028913194221461</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>42.48192274653715</v>
+        <v>42.48192271990463</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>30.04794274966148</v>
+        <v>30.04794246560368</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.2501599396096814</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-1.291802676947541</v>
+        <v>-1.291802676415414</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>619.4782183600228</v>
+        <v>619.4782183600238</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>472</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>55.82687224204486</v>
+        <v>55.82687234176015</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>22.08385971397313</v>
+        <v>22.08385990619946</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.865041219778342</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>4.10893205517692</v>
+        <v>4.108932051413049</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>610.6013962923112</v>
+        <v>610.6013962923113</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>50</v>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>61.7646697223823</v>
+        <v>61.76466998866634</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>25.2116578831926</v>
+        <v>25.21165818000409</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.140741378769861</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.07249027042325401</v>
+        <v>0.07249027016367782</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>50.40165483345383</v>
+        <v>50.40165487128143</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>26.14804709642917</v>
+        <v>26.14804729550728</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.5791253972083167</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-1.693799943306909</v>
+        <v>-1.693799944578823</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>577.4650523533123</v>
+        <v>577.4650523533122</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>597</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>50.72621450008403</v>
+        <v>50.72621446759339</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>31.53902368895329</v>
+        <v>31.53902381118123</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.4832205599883757</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-8.311415719534434</v>
+        <v>-8.311415718366369</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>571.9514534984928</v>
+        <v>571.9514534984929</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>19.55</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>52.29308520893061</v>
+        <v>52.29308520366342</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>7.38586692747694</v>
+        <v>7.385866887955562</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.9435408730111927</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.3680997728875546</v>
+        <v>0.368099772991384</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>571.7477354972317</v>
+        <v>571.7477354972316</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>232</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>42.43749228234979</v>
+        <v>42.43749229197072</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>28.93118720321106</v>
+        <v>28.93118721219972</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.5603887573874565</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-5.813970493924819</v>
+        <v>-5.813970494418005</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>60.52530551074071</v>
+        <v>60.52530552710639</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>31.63464733604794</v>
+        <v>31.63464738002723</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>2.53425075941183</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-5.099216836016609</v>
+        <v>-5.099216838482505</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>66.95384630257544</v>
+        <v>66.95384635554649</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>36.24106969199593</v>
+        <v>36.24106969201431</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>13.57004154429711</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.280897501275817</v>
+        <v>1.280897501444539</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>558.1509004929644</v>
+        <v>558.1509004929636</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>115</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>58.25200564476405</v>
+        <v>58.25200599885891</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>23.8649010645223</v>
+        <v>23.86490113444244</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.29480849990638</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.46874137484461</v>
+        <v>0.4687413739361129</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>548.2128851983215</v>
+        <v>548.2128851983216</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>41.85</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>43.48960106896989</v>
+        <v>43.48960113609603</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>21.20336229737828</v>
+        <v>21.20336236407856</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>2.152664272709147</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.4155686625625881</v>
+        <v>0.415568662340154</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>43.96007259048138</v>
+        <v>43.96007258936589</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>36.05988863148296</v>
+        <v>36.0598886415957</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5113305909110898</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-1.20503810805427</v>
+        <v>-1.205038108072437</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>45.18736472900692</v>
+        <v>45.18736474461694</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>22.21152687383203</v>
+        <v>22.21152693855917</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.7864727676954077</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-6.192578774217576</v>
+        <v>-6.192578775255869</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         <v>43.41363655403386</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>20.82924988418803</v>
+        <v>20.82925010494149</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.1866793272497344</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.7767470553439226</v>
+        <v>-0.7767470555385939</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>493.2204727641994</v>
+        <v>493.2204727641995</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>104.5</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>50.04581624807792</v>
+        <v>50.04581625924752</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24.01983924377861</v>
+        <v>24.01983942891731</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.4830325583215399</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-1.378983245600434</v>
+        <v>-1.378983244925559</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>56.53966589481185</v>
+        <v>56.53966589134033</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.24587084498942</v>
+        <v>31.24587078004762</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.3407759209715591</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.1250449838521526</v>
+        <v>0.1250449840208798</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>487.2097275784325</v>
+        <v>487.2097275784323</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>46</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.32572715890439</v>
+        <v>57.32572722921451</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>40.65618556437843</v>
+        <v>40.65618557774729</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.8579285059578369</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.1599100456371082</v>
+        <v>0.1599100455332787</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>43.43573046159274</v>
+        <v>43.43573050919412</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>10.92814114056611</v>
+        <v>10.92814117291418</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6308991060770219</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>3.220756256699413</v>
+        <v>3.220756256180326</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>41.01842364847722</v>
+        <v>41.01842365791195</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>22.25653640119004</v>
+        <v>22.25653663076563</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.7881131899594851</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-3.016949127973012</v>
+        <v>-3.016949128362338</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>45.64879485948919</v>
+        <v>45.64879488325099</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>26.36145669580239</v>
+        <v>26.36145686716847</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.6606877362996376</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.5764223441692444</v>
+        <v>-0.5764223443898869</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>44.38903008910564</v>
+        <v>44.38903008640304</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>24.47871259229134</v>
+        <v>24.47871251068761</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.4188212073909783</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-1.497159607456259</v>
+        <v>-1.497159607495197</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>51.99799419613434</v>
+        <v>51.9979942215828</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.03045116843188</v>
+        <v>28.03045122781381</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.8073056122401421</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.3724378738241652</v>
+        <v>-0.3724378742135421</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>451.6897327308894</v>
+        <v>451.6897327308895</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>317</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>43.03512729454533</v>
+        <v>43.03512732561887</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>22.96535417764487</v>
+        <v>22.96535419368785</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.743549978550329</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-5.526473731241047</v>
+        <v>-5.526473732019731</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>448.7890260317169</v>
+        <v>448.789026031717</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>18.85</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>54.17252468642187</v>
+        <v>54.17252476598073</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>6.465255335144739</v>
+        <v>6.465255837183021</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.4978017104403912</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.003570395288495787</v>
+        <v>-0.003570395574027052</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>30.97607550061628</v>
+        <v>30.97607562471484</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>29.10603318326356</v>
+        <v>29.1060332513963</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4070879222902932</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-11.86443332235417</v>
+        <v>-11.864433325469</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>443.2818300350433</v>
+        <v>443.2818300350431</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>910</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>51.47606461986035</v>
+        <v>51.47606460457181</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>15.70882893857922</v>
+        <v>15.70882899671447</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7153998161566312</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>6.120000213229346</v>
+        <v>6.120000208557011</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>43.07001023667062</v>
+        <v>43.07001024196642</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.31186054987297</v>
+        <v>20.31186077810607</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.7271413870251814</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.6595038249322008</v>
+        <v>-0.6595038251268825</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>425.7006018832118</v>
+        <v>425.7006018832119</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>96.3</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>43.07267987866539</v>
+        <v>43.07267998026353</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>16.10236338725004</v>
+        <v>16.10236348642621</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8213115440132339</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.6177699439458755</v>
+        <v>-0.6177699451139422</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>29.0488010639813</v>
+        <v>29.04880106999937</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>24.00473785967107</v>
+        <v>24.0047379485804</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.4395881901848726</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-2.287462812053302</v>
+        <v>-2.287462812416705</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>422.409709494459</v>
+        <v>422.4097094944597</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>21.2</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>39.33646446054198</v>
+        <v>39.33646449845289</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>15.1739034166078</v>
+        <v>15.17390352224302</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.7280176980431818</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.1138734202031115</v>
+        <v>-0.1138734203328983</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>419.5225993511321</v>
+        <v>419.5225993511318</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>12.4</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>48.26300861798374</v>
+        <v>48.26300868512116</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>31.6518677951872</v>
+        <v>31.65186784950163</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.577254236615266</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.05353483125443645</v>
+        <v>-0.05353483134528794</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>40.20477865001131</v>
+        <v>40.20477836627167</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>25.52246550091668</v>
+        <v>25.52246566965961</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4165843898479347</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-2.115153760662388</v>
+        <v>-2.115153758404115</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>43.6231682260992</v>
+        <v>43.62316828151636</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>21.6859000493734</v>
+        <v>21.68590023469326</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5971790049014803</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.982313014288239</v>
+        <v>-1.982313017273315</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>390.3716792665684</v>
+        <v>390.3716792665695</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>66.40000000000001</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>36.51630034547541</v>
+        <v>36.5163003784789</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>17.05801338360466</v>
+        <v>17.05801356902393</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.6658116057695529</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.7485696728379544</v>
+        <v>-0.7485696732402938</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>387.7442054053454</v>
+        <v>387.7442054053459</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>64.7</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>35.69826603924925</v>
+        <v>35.69826600268608</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.2042564816358</v>
+        <v>22.20425659630393</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6613033381130128</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-1.095400227601492</v>
+        <v>-1.095400227653411</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>49.63021911942405</v>
+        <v>49.63021895151141</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>13.52333650413539</v>
+        <v>13.52333661687568</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5770372728174034</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.1053667728442537</v>
+        <v>0.1053667728702124</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>42.46093498776879</v>
+        <v>42.46093502926755</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>22.68086867198395</v>
+        <v>22.68086874762121</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.209624947391127</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-1.472203857415822</v>
+        <v>-1.472203858713728</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>48.88100527977116</v>
+        <v>48.88100525967484</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.42720932304584</v>
+        <v>11.42720954479049</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.8040499993026722</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.1525767164610537</v>
+        <v>-0.1525767165778569</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>48.71126878500866</v>
+        <v>48.71126886024458</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>19.71376689412944</v>
+        <v>19.71376691315064</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.5190079314417678</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.02471207152306019</v>
+        <v>0.02471207143220994</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>362.1305553446718</v>
+        <v>362.1305553446717</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>49.3</v>
@@ -3470,7 +3470,7 @@
         <v>46.96597950069045</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>17.75779138407032</v>
+        <v>17.75779143753459</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.504251063292833</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.9111276447059731</v>
+        <v>-0.9111276447319314</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>359.8901219766541</v>
+        <v>359.8901219766542</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1260</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>41.98032748303256</v>
+        <v>41.9803274788225</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.61668686202148</v>
+        <v>23.61668679874655</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.6588398461457313</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-28.88229394137132</v>
+        <v>-28.88229394266896</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>358.1073475243682</v>
+        <v>358.1073475243697</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>40.5</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>42.34963721468672</v>
+        <v>42.3496372319269</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.04113878467574</v>
+        <v>20.04113881620643</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.7065556234253727</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.3333043152307572</v>
+        <v>-0.3333043153864979</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>45.09504438757064</v>
+        <v>45.09504446452429</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>23.82667909218408</v>
+        <v>23.82667916190858</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.176351588861237</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>39.29259755407259</v>
+        <v>39.2925975933078</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>18.12821706298998</v>
+        <v>18.12821706449261</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.9505886200777706</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.01006520375479891</v>
+        <v>0.01006520370288294</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         <v>42.67162790447533</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>15.80925979190588</v>
+        <v>15.80925978272022</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.720218977300666</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-1.450102454800556</v>
+        <v>-1.450102454787583</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.06658272241659</v>
+        <v>44.06658278474664</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.80406053988675</v>
+        <v>23.80406055080532</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3986958506219546</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.01881207816714953</v>
+        <v>0.0188120780633162</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>342.5937962191653</v>
+        <v>342.5937962191654</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>21.45</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>41.08666675541784</v>
+        <v>41.08666673932102</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>12.00186828898663</v>
+        <v>12.0018683298396</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.3186330594557458</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.194794316305846</v>
+        <v>-0.1947943164356323</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>338.7687621748494</v>
+        <v>338.7687621748493</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>54.3</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>40.60047022560941</v>
+        <v>40.60047027464629</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>12.96595014738856</v>
+        <v>12.96595018636582</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.4458939642293094</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.4713973299976539</v>
+        <v>-0.4713973303740281</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>36.48514492491609</v>
+        <v>36.48514494369422</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>20.51815875354233</v>
+        <v>20.51815889733559</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.7673668027537495</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-4.996363063603033</v>
+        <v>-4.996363064771156</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>332.0092306554644</v>
+        <v>332.0092306554643</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>45.25</v>
@@ -4000,7 +4000,7 @@
         <v>40.93190921581994</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>9.750587254043181</v>
+        <v>9.750587199300613</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4426821867782229</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.02268243934997183</v>
+        <v>-0.02268243914230822</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>328.483412616205</v>
+        <v>328.4834126162063</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>41.7</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.30688813253867</v>
+        <v>42.30688816675527</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>15.29926197787438</v>
+        <v>15.29926213219526</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.6291091592888773</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.1351173205114093</v>
+        <v>-0.1351173207320366</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>43.57309485663201</v>
+        <v>43.57309476926993</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.28813049923044</v>
+        <v>15.28813054035275</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3142562496879532</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.8109780197796138</v>
+        <v>-0.8109780195459975</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4159,7 +4159,7 @@
         <v>32.03038264205276</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>24.49085421151782</v>
+        <v>24.49085424502265</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.58591246754207</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.2211326876192501</v>
+        <v>-0.2211326876452091</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>60.8538244503473</v>
+        <v>60.85382488330799</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>19.37674902823226</v>
+        <v>19.37674930391606</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.8343576285214932</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.09831599355995868</v>
+        <v>0.09831599333123497</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>37.92822107307615</v>
+        <v>37.92822110967214</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.45138754352809</v>
+        <v>22.45138767198857</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.8133622177079534</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-5.147699664849853</v>
+        <v>-5.147699666147743</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>43.75573262096812</v>
+        <v>43.7557326243288</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.87684334603674</v>
+        <v>14.87684339446275</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.6373885306045443</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.2644615532043315</v>
+        <v>-0.2644615532173088</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>317.622669790989</v>
+        <v>317.6226697909884</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>23.2</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>42.54610965218362</v>
+        <v>42.54610963574236</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.49868882289624</v>
+        <v>14.49868891398552</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.7337116262418329</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.06644144035911062</v>
+        <v>-0.06644144042400554</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>34.96580266540288</v>
+        <v>34.96580267047571</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>20.09652617965135</v>
+        <v>20.09652617979782</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.934941983401482</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.2357764095016</v>
+        <v>46.23577657025787</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>9.103864300988578</v>
+        <v>9.103864503199361</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.560135065854949</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1214513120895138</v>
+        <v>-0.1214513132016611</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.22630981074426</v>
+        <v>52.22630981911153</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>13.04338907658055</v>
+        <v>13.04338897257761</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4506725487651918</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.4440891499067408</v>
+        <v>-0.444089150789291</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>311.9804891749344</v>
+        <v>311.9804891749366</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>50.5</v>
@@ -4580,7 +4580,7 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>38.12016307802378</v>
+        <v>38.12016304578459</v>
       </c>
       <c r="I78" s="2" t="n">
         <v>6.852570144367955</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.02594204657897616</v>
+        <v>-0.02594204660493094</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>37.21330452121752</v>
+        <v>37.21330444108085</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>9.465805361857504</v>
+        <v>9.465805422527808</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.9879476334987756</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.268027523786165</v>
+        <v>-0.2680275236563803</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>48.09318554494792</v>
+        <v>48.09318561686796</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>15.26455533968555</v>
+        <v>15.26455533280837</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.6080695334232654</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.06866616039812959</v>
+        <v>-0.06866616052791649</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>42.2626352290009</v>
+        <v>42.26263508135629</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>13.4820941020908</v>
+        <v>13.48209430188449</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.5314520845681304</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.131168746574325</v>
+        <v>-0.1311687464445384</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>282.2519713292633</v>
+        <v>282.251971329263</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>97.3</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>33.00668851463618</v>
+        <v>33.0066884658544</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.51638197675785</v>
+        <v>27.51638200017733</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.513697526763331</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>39.63647650673768</v>
+        <v>39.636476738601</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>29.14200501989702</v>
+        <v>29.14200504635948</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.7055078030690214</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-1.92155246902073</v>
+        <v>-1.92155247161646</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>275.8955318291406</v>
+        <v>275.8955318291405</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>213</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>32.17204048878885</v>
+        <v>32.17204049819425</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>18.61855943002146</v>
+        <v>18.61855957768476</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.4418196652627401</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-4.277029716987982</v>
+        <v>-4.277029717507125</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>39.74253342036971</v>
+        <v>39.7425334334281</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>19.82601702725682</v>
+        <v>19.82601724467363</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.730924899218151</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-30.57943229977781</v>
+        <v>-30.57943230678627</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>266.4868197135004</v>
+        <v>266.4868197135008</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>72.3</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>38.50361059488515</v>
+        <v>38.50361059945103</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>16.77364682839044</v>
+        <v>16.77364683899512</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.6177546508757084</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.3803953203069896</v>
+        <v>-0.3803953205665522</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>38.74714828117263</v>
+        <v>38.74714832246571</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>22.87808888526706</v>
+        <v>22.87808890839352</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.031704685850572</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.1915744317372401</v>
+        <v>-0.1915744321265964</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>48.15529524225773</v>
+        <v>48.15529523425525</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>19.7107992943572</v>
+        <v>19.71079933393996</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.649037471566105</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.1667650627196914</v>
+        <v>-0.1667650628364989</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>37.1635754371842</v>
+        <v>37.16357542663297</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>16.87350913251257</v>
+        <v>16.87350930133317</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.6220159686264627</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.2109864397510212</v>
+        <v>-0.2109864397250648</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>40.77252138030745</v>
+        <v>40.77252145651015</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>21.96379934198058</v>
+        <v>21.96379936653261</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.4918371564372804</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.0155764033596959</v>
+        <v>-0.01557640348948058</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>44.55140989863094</v>
+        <v>44.55140987825153</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>13.96089785711258</v>
+        <v>13.96089788036257</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-1.425587248421056</v>
+        <v>-1.425587248291268</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>237.8816705887379</v>
+        <v>237.881670588738</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>127.5</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>34.91987974041824</v>
+        <v>34.9198795097312</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>12.97696194553589</v>
+        <v>12.97696206154622</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.8352331012409452</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.8782033300950001</v>
+        <v>-0.8782033290567237</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>234.2400448020725</v>
+        <v>234.2400448020724</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>89.2</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.12404507175991</v>
+        <v>35.12404480539568</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.93071925057663</v>
+        <v>17.93071944941106</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.9621708467024712</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.4948365691088927</v>
+        <v>-0.4948365706663271</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>39.68120852153761</v>
+        <v>39.68120863300165</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>13.54440823327485</v>
+        <v>13.54440825772829</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.8367183991488116</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.4773424464668279</v>
+        <v>-0.4773424468042709</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>42.40987571441958</v>
+        <v>42.40987572787235</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>18.66631841803529</v>
+        <v>18.66631845639528</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.2388615937016738</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.6066177946077824</v>
+        <v>-0.6066177946856586</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>36.33721909298977</v>
+        <v>36.33721909884041</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>11.89911395834071</v>
+        <v>11.89911400838402</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.7088647421102982</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>41.04106358117504</v>
+        <v>41.04106353926579</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.54458384347341</v>
+        <v>14.5445837894609</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.5793334974259351</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-1.794214876103579</v>
+        <v>-1.794214876882355</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>220.8907140876711</v>
+        <v>220.8907140876718</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>48.2</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.72261137385655</v>
+        <v>42.72261151552643</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.4402820444486</v>
+        <v>19.44028203172052</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.6455369966166463</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.2127286602613465</v>
+        <v>-0.2127286604690019</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>40.68829055885323</v>
+        <v>40.68829056401932</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>19.30406044905748</v>
+        <v>19.30406058612635</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.3277851763556027</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-2.662322785809681</v>
+        <v>-2.662322785978386</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>39.87430339923723</v>
+        <v>39.87430340127597</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>16.07269091723709</v>
+        <v>16.0726909347484</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.732448737896305</v>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>213.992578252269</v>
+        <v>213.9925782522706</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>35.45</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>36.64448632843487</v>
+        <v>36.64448647962521</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>16.00795412429219</v>
+        <v>16.00795407161245</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.5427307671178602</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.1323493480862767</v>
+        <v>-0.1323493481122316</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.74412485819607</v>
+        <v>41.7441248890414</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>16.10483769542439</v>
+        <v>16.10483790391011</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.4215792906941168</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.1021127027909715</v>
+        <v>-0.102112702959697</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         <v>38.75829517534873</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.03675796292755</v>
+        <v>12.03675806765995</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.4552798044629044</v>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>196.8052914312745</v>
+        <v>196.8052914312746</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>61</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>40.18137479973824</v>
+        <v>40.18137515989376</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>21.9304835296479</v>
+        <v>21.93048348874958</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.02958028798918</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.05609541111465222</v>
+        <v>0.05609540916784084</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>171.8923795645469</v>
+        <v>171.8923795645468</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>23.2</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>37.01438917751854</v>
+        <v>37.01438772758838</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.16633910633625</v>
+        <v>18.16634082012416</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.173065588498997</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.1595868411806254</v>
+        <v>-0.1595868389223357</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>171.738977737577</v>
+        <v>171.7389777375785</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>108</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>43.0796834240035</v>
+        <v>43.07968354876465</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.12535511014446</v>
+        <v>16.12535518403117</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.491893028793488</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.5333153709764629</v>
+        <v>-0.5333153720147675</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>47.70824979176303</v>
+        <v>47.70825010650694</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>11.32705224788188</v>
+        <v>11.32705217296843</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.7033086634740966</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.06779734638887819</v>
+        <v>0.06779734590866815</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>39.04530017218787</v>
+        <v>39.04530025725249</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>18.20537904403647</v>
+        <v>18.20537912989366</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6093792743911375</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-25.85459688399067</v>
+        <v>-25.85459688476932</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>136.2855693354552</v>
+        <v>136.2855693354545</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>32.25</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>38.0311444233766</v>
+        <v>38.03114515793416</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.87114521283742</v>
+        <v>18.87114529187345</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.2637962126132823</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.2893208648187467</v>
+        <v>-0.2893208650783236</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>39.42928373469721</v>
+        <v>39.4292838588584</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>21.49564502326353</v>
+        <v>21.49564508367213</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.235452198499643</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.2875912621471023</v>
+        <v>-0.2875912624975255</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>41.00225268692087</v>
+        <v>41.00225265806684</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.92605785373228</v>
+        <v>18.92605770829745</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.501698398289172</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-2.423439907959115</v>
+        <v>-2.423439907504846</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>116.1812168088303</v>
+        <v>116.1812168088304</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>45.7</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>31.76191439235775</v>
+        <v>31.76191441561846</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>11.60455401121164</v>
+        <v>11.60455407689306</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>1.186004476211294</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.2726743076077329</v>
+        <v>-0.2726743077764512</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>106.2281384094418</v>
+        <v>106.2281384094414</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>18.5</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>49.17189697070339</v>
+        <v>49.17189695544685</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>6.53771727056706</v>
+        <v>6.537717299968499</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.762763858258577</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.02907943209277046</v>
+        <v>0.02907943214468557</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>57.88731979447381</v>
+        <v>57.88731979447366</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>72.3</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>35.16830352376803</v>
+        <v>35.16830381854814</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>15.57303903348749</v>
+        <v>15.5730388209383</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>1.155096072214059</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.06504822902631313</v>
+        <v>0.06504822850717429</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>40.45289783597476</v>
+        <v>40.45289783597504</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>56.5</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>22.82307696936611</v>
+        <v>22.82307701330924</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>16.14584122399383</v>
+        <v>16.14584114068564</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.6973022282200585</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.2827038228541241</v>
+        <v>-0.2827038231396533</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>21.31005534658614</v>
+        <v>21.31005534658615</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>17.95</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>48.5124896867868</v>
+        <v>48.51248972795864</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>9.310229972946777</v>
+        <v>9.310229865554501</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.1556555978811549</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.08810602397990547</v>
+        <v>0.0881060235645888</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg5 2026-10-27 00:08 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq6_2026-10-22.xlsx
@@ -444,7 +444,7 @@
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>78.90131156175438</v>
+        <v>78.901311650401</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>33.15849061754602</v>
+        <v>33.15849069222572</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.887832827195892</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.1917634640524146</v>
+        <v>0.191763463912249</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>88.80743663051797</v>
+        <v>88.80743663339511</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>40.42124236999416</v>
+        <v>40.42124235158894</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>4.685271930498494</v>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>67.03613243533684</v>
+        <v>67.03613181539461</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>19.45238169571356</v>
+        <v>19.45238179633244</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.026592574560778</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.04737782209310933</v>
+        <v>0.04737782212114357</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65.6407222068942</v>
+        <v>65.64072225781808</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>34.89015513951923</v>
+        <v>34.8901552567762</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.416036974209795</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-0.3201726229496833</v>
+        <v>-0.3201726228095172</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>55.0856830495019</v>
+        <v>55.08568306302619</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>36.65148684351382</v>
+        <v>36.65148697570977</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.233027650764054</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>-5.186169113878286</v>
+        <v>-5.186169114262666</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>857.2373126052629</v>
+        <v>857.2373126052628</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>90.09999999999999</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.41895069619824</v>
+        <v>60.41895152803244</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>33.02733246566626</v>
+        <v>33.02733296206482</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.281559472437751</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.02741526840408426</v>
+        <v>0.02741526644170511</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>54.64295263835304</v>
+        <v>54.64295267003019</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>33.47085421456798</v>
+        <v>33.47085420987621</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.6145525805647692</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-0.6052151005438731</v>
+        <v>-0.6052151007120763</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>66.14815023444106</v>
+        <v>66.14815027975249</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>33.13629602100019</v>
+        <v>33.13629602271578</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2.544511166061138</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.7480122021666666</v>
+        <v>0.7480122020405191</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>60.06618490310662</v>
+        <v>60.06618492723181</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>49.94953734204721</v>
+        <v>49.94953748794686</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.398229788631511</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.547504950749008</v>
+        <v>1.547504950678921</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>59.64192344313563</v>
+        <v>59.64192350656069</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>26.41004659100323</v>
+        <v>26.41004665243693</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>3.166044129630837</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>2.003902512580358</v>
+        <v>2.00390251196362</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>712.1949567710933</v>
+        <v>712.1949567710934</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>26.85</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>82.00485241673489</v>
+        <v>82.00485252903977</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>52.30388558433571</v>
+        <v>52.30388560759321</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>2.033008627467827</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.2300014569881352</v>
+        <v>0.2300014569320661</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>49.94045106699661</v>
+        <v>49.94045126700379</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>36.37853757561509</v>
+        <v>36.37853763934768</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.6998040680600051</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-0.9585343487223748</v>
+        <v>-0.9585343506847472</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>677.0219967973212</v>
+        <v>677.0219967973214</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>45.9</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>68.14931598112399</v>
+        <v>68.14931621063776</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>35.44148194933189</v>
+        <v>35.44148200241577</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.6476559223050367</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.2317171873639329</v>
+        <v>0.2317171871396633</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>673.8203676915855</v>
+        <v>673.8203676915966</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>32.6</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>69.44974491603531</v>
+        <v>69.4497452865578</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>41.35617015557782</v>
+        <v>41.35617013089941</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>5.971524141804417</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.07751029840802381</v>
+        <v>0.07751029816973354</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>64.81172467745395</v>
+        <v>64.81172469291985</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>51.3059022253042</v>
+        <v>51.30590226155739</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.252859594182261</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3.795119547750986</v>
+        <v>3.79511954747063</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>640.8772581040774</v>
+        <v>640.8772581040773</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>89.8</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>53.90440152316441</v>
+        <v>53.90440182572696</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>28.80512429673319</v>
+        <v>28.80512431046055</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.6183082921517314</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.1028913194221461</v>
+        <v>0.1028913205434878</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>42.48192271990463</v>
+        <v>42.4819225802676</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>30.04794246560368</v>
+        <v>30.0479422159358</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.2501599396096814</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-1.291802676415414</v>
+        <v>-1.291802675966877</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>619.4782183600238</v>
+        <v>619.478218360023</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>472</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>55.82687234176015</v>
+        <v>55.82687230544324</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>22.08385990619946</v>
+        <v>22.08385989167767</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.865041219778342</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>4.108932051413049</v>
+        <v>4.108932053235302</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>610.6013962923113</v>
+        <v>610.6013962923114</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>50</v>
@@ -1509,7 +1509,7 @@
         <v>61.76466998866634</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>25.21165818000409</v>
+        <v>25.21165813999458</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.140741378769861</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>50.40165487128143</v>
+        <v>50.40165490756138</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>26.14804729550728</v>
+        <v>26.14804748521312</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.5791253972083167</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-1.693799944578823</v>
+        <v>-1.693799945167536</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>50.72621446759339</v>
+        <v>50.72621449826526</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>31.53902381118123</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-8.311415718366369</v>
+        <v>-8.311415719347643</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>52.29308520366342</v>
+        <v>52.29308520662966</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>7.385866887955562</v>
+        <v>7.38586689999112</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.9435408730111927</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.368099772991384</v>
+        <v>0.3680997728792484</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>42.43749229197072</v>
+        <v>42.43749232377858</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>28.93118721219972</v>
+        <v>28.9311873203415</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.5603887573874565</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-5.813970494418005</v>
+        <v>-5.813970494558173</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>60.52530552710639</v>
+        <v>60.5253055440927</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>31.63464738002723</v>
+        <v>31.63464752250954</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>2.53425075941183</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-5.099216838482505</v>
+        <v>-5.099216839463779</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>66.95384635554649</v>
+        <v>66.95384638707176</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>36.24106969201431</v>
+        <v>36.24106969418396</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>13.57004154429711</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.280897501444539</v>
+        <v>1.280897502159402</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>558.1509004929636</v>
+        <v>558.1509004929643</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>115</v>
@@ -1880,7 +1880,7 @@
         <v>58.25200599885891</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>23.86490113444244</v>
+        <v>23.86490113878756</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.29480849990638</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.4687413739361129</v>
+        <v>0.4687413742164473</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>43.48960113609603</v>
+        <v>43.48960112933737</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>21.20336236407856</v>
+        <v>21.2033623532975</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>2.152664272709147</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.415568662340154</v>
+        <v>0.4155686624122242</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>43.96007258936589</v>
+        <v>43.96007259541209</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>36.0598886415957</v>
+        <v>36.05988865340181</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5113305909110898</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-1.205038108072437</v>
+        <v>-1.205038108100469</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>45.18736474461694</v>
+        <v>45.18736474405657</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>22.21152693855917</v>
+        <v>22.21152701898373</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.7864727676954077</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-6.192578775255869</v>
+        <v>-6.192578775536179</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>43.41363655403386</v>
+        <v>43.41363661848646</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>20.82925010494149</v>
+        <v>20.82925006630665</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.1866793272497344</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.7767470555385939</v>
+        <v>-0.7767470557488475</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>493.2204727641995</v>
+        <v>493.2204727641996</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>104.5</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>50.04581625924752</v>
+        <v>50.04581616094982</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24.01983942891731</v>
+        <v>24.01983941284163</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.4830325583215399</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-1.378983244925559</v>
+        <v>-1.378983244028463</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>56.53966589134033</v>
+        <v>56.53966588171265</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>31.24587078004762</v>
+        <v>31.24587079558084</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.3407759209715591</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.1250449840208798</v>
+        <v>0.1250449841470225</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.32572722921451</v>
+        <v>57.32572725445404</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>40.65618557774729</v>
+        <v>40.65618564660782</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.8579285059578369</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.1599100455332787</v>
+        <v>0.159910045505243</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>43.43573050919412</v>
+        <v>43.43573047366545</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>10.92814117291418</v>
+        <v>10.92814104955457</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6308991060770219</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>3.220756256180326</v>
+        <v>3.220756260805814</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>41.01842365791195</v>
+        <v>41.01842369221229</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>22.25653663076563</v>
+        <v>22.25653665270901</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.7881131899594851</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-3.016949128362338</v>
+        <v>-3.016949128502516</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>45.64879488325099</v>
+        <v>45.64879489604579</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>26.36145686716847</v>
+        <v>26.36145702610619</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.6606877362996376</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.5764223443898869</v>
+        <v>-0.5764223444879946</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>44.38903008640304</v>
+        <v>44.38903009914875</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>24.47871251068761</v>
+        <v>24.47871255214793</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.4188212073909783</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-1.497159607495197</v>
+        <v>-1.497159607565285</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>51.9979942215828</v>
+        <v>51.99799423528582</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.03045122781381</v>
+        <v>28.03045121788873</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.8073056122401421</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.3724378742135421</v>
+        <v>-0.3724378743537136</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>451.6897327308895</v>
+        <v>451.6897327308894</v>
       </c>
       <c r="E40" s="2" t="n">
         <v>317</v>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>43.03512732561887</v>
+        <v>43.03512732954065</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>22.96535419368785</v>
+        <v>22.96535423670838</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.743549978550329</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-5.526473732019731</v>
+        <v>-5.526473731459085</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>448.789026031717</v>
+        <v>448.7890260317168</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>18.85</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>54.17252476598073</v>
+        <v>54.1725247833237</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>6.465255837183021</v>
+        <v>6.465255830240836</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.4978017104403912</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.003570395574027052</v>
+        <v>-0.003570395616077082</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>30.97607562471484</v>
+        <v>30.97607563505603</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>29.1060332513963</v>
+        <v>29.10603323831181</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4070879222902932</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-11.864433325469</v>
+        <v>-11.8644333215443</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>443.2818300350431</v>
+        <v>443.2818300350429</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>910</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>51.47606460457181</v>
+        <v>51.47606490853165</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>15.70882899671447</v>
+        <v>15.7088290677179</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7153998161566312</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>6.120000208557011</v>
+        <v>6.120000202389516</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>43.07001024196642</v>
+        <v>43.07001028968867</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>20.31186077810607</v>
+        <v>20.31186084108358</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.7271413870251814</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.6595038251268825</v>
+        <v>-0.6595038252810588</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>425.7006018832119</v>
+        <v>425.700601883212</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>96.3</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>43.07267998026353</v>
+        <v>43.07268021240122</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>16.10236348642621</v>
+        <v>16.10236351986086</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8213115440132339</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.6177699451139422</v>
+        <v>-0.6177699456746359</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>425.3396473012075</v>
+        <v>425.3396473012078</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>103.5</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>29.04880106999937</v>
+        <v>29.04880107972087</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>24.0047379485804</v>
+        <v>24.00473798756883</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.4395881901848726</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-2.287462812416705</v>
+        <v>-2.287462812697045</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>422.4097094944597</v>
+        <v>422.4097094944589</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>21.2</v>
@@ -2940,7 +2940,7 @@
         <v>39.33646449845289</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>15.17390352224302</v>
+        <v>15.17390364062785</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.7280176980431818</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.1138734203328983</v>
+        <v>-0.1138734203749517</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>48.26300868512116</v>
+        <v>48.26300871833809</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>31.65186784950163</v>
+        <v>31.65186787716851</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.577254236615266</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>40.20477836627167</v>
+        <v>40.20477840928482</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>25.52246566965961</v>
+        <v>25.52246586417724</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4165843898479347</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-2.115153758404115</v>
+        <v>-2.115153759357254</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>43.62316828151636</v>
+        <v>43.62316830666394</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>21.68590023469326</v>
+        <v>21.68590035780623</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5971790049014803</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.982313017273315</v>
+        <v>-1.982313017974166</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>390.3716792665695</v>
+        <v>390.3716792665684</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>66.40000000000001</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>36.5163003784789</v>
+        <v>36.51630040431031</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>17.05801356902393</v>
+        <v>17.05801364001351</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.6658116057695529</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.7485696732402938</v>
+        <v>-0.7485696733243925</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>387.7442054053459</v>
+        <v>387.7442054053425</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>64.7</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>35.69826600268608</v>
+        <v>35.69826603385852</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.20425659630393</v>
+        <v>22.20425660015665</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6613033381130128</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-1.095400227653411</v>
+        <v>-1.095400228045884</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>49.63021895151141</v>
+        <v>49.63021908967129</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>13.52333661687568</v>
+        <v>13.52333669288898</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5770372728174034</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.1053667728702124</v>
+        <v>0.1053667724216608</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>42.46093502926755</v>
+        <v>42.46093504137975</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>22.68086874762121</v>
+        <v>22.68086876616175</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.209624947391127</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>48.88100525967484</v>
+        <v>48.88100534147562</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>11.42720954479049</v>
+        <v>11.42720962895418</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.8040499993026722</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.1525767165778569</v>
+        <v>-0.1525767168021311</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>48.71126886024458</v>
+        <v>48.71126890971599</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>19.71376691315064</v>
+        <v>19.7137669221596</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.5190079314417678</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.02471207143220994</v>
+        <v>0.0247120714041755</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>362.1305553446717</v>
+        <v>362.1305553446718</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>49.3</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>46.96597950069045</v>
+        <v>46.96597950348534</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>17.75779143753459</v>
+        <v>17.75779144220804</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.504251063292833</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.9111276447319314</v>
+        <v>-0.9111276447599703</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>359.8901219766542</v>
+        <v>359.8901219766538</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1260</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>41.9803274788225</v>
+        <v>41.98032749528994</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.61668679874655</v>
+        <v>23.61668686191035</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.6588398461457313</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-28.88229394266896</v>
+        <v>-28.88229394519234</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>358.1073475243697</v>
+        <v>358.1073475243678</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>40.5</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>42.3496372319269</v>
+        <v>42.3496372579198</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>20.04113881620643</v>
+        <v>20.04113881941166</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.7065556234253727</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.3333043153864979</v>
+        <v>-0.333304315484624</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>45.09504446452429</v>
+        <v>45.09504468261159</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>23.82667916190858</v>
+        <v>23.82667923723947</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.176351588861237</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-6.293124571423642</v>
+        <v>-6.293124568760396</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>352.6703790402014</v>
+        <v>352.6703790402013</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>39.75</v>
@@ -3682,7 +3682,7 @@
         <v>39.2925975933078</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>18.12821706449261</v>
+        <v>18.12821702997862</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.9505886200777706</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.01006520370288294</v>
+        <v>0.01006520367485725</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>42.67162790447533</v>
+        <v>42.67162789016278</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>15.80925978272022</v>
+        <v>15.80925958917357</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.720218977300666</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-1.450102454787583</v>
+        <v>-1.45010245477356</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>44.06658278474664</v>
+        <v>44.06658274309965</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.80406055080532</v>
+        <v>23.80406054722563</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3986958506219546</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0188120780633162</v>
+        <v>0.01881207809134067</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>342.5937962191654</v>
+        <v>342.5937962191653</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>21.45</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>41.08666673932102</v>
+        <v>41.08666680288282</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>12.0018683298396</v>
+        <v>12.00186851463728</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.3186330594557458</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1947943164356323</v>
+        <v>-0.194794316617853</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>338.7687621748493</v>
+        <v>338.7687621748494</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>54.3</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>40.60047027464629</v>
+        <v>40.60047036519811</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>12.96595018636582</v>
+        <v>12.9659502304512</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.4458939642293094</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.4713973303740281</v>
+        <v>-0.4713973304721505</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>36.48514494369422</v>
+        <v>36.48514492911995</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>20.51815889733559</v>
+        <v>20.51815898728553</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.7673668027537495</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-4.996363064771156</v>
+        <v>-4.99636306463097</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>40.93190921581994</v>
+        <v>40.93190904364949</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>9.750587199300613</v>
+        <v>9.750586983917623</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4426821867782229</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.02268243914230822</v>
+        <v>-0.02268243891803745</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.30688816675527</v>
+        <v>42.30688822339985</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>15.29926213219526</v>
+        <v>15.29926216213074</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.6291091592888773</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.1351173207320366</v>
+        <v>-0.1351173208161472</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>43.57309476926993</v>
+        <v>43.57309488806039</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>15.28813054035275</v>
+        <v>15.28813049515237</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3142562496879532</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.8109780195459975</v>
+        <v>-0.8109780199104366</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>32.03038264205276</v>
+        <v>32.03038265836361</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>24.49085424502265</v>
+        <v>24.4908542707221</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.58591246754207</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.2211326876452091</v>
+        <v>-0.221132687673246</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>60.85382488330799</v>
+        <v>60.85382493329802</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>19.37674930391606</v>
+        <v>19.37674946537529</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.8343576285214932</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>37.92822110967214</v>
+        <v>37.92822120389889</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>22.45138767198857</v>
+        <v>22.45138783321344</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.8133622177079534</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-5.147699666147743</v>
+        <v>-5.147699666007562</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4318,7 +4318,7 @@
         <v>43.7557326243288</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.87684339446275</v>
+        <v>14.87684335649412</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.6373885306045443</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>42.54610963574236</v>
+        <v>42.54610978979809</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.49868891398552</v>
+        <v>14.49868898414089</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.7337116262418329</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.06644144042400554</v>
+        <v>-0.06644144050810967</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>34.96580267047571</v>
+        <v>34.96580266501265</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>20.09652617979782</v>
+        <v>20.09652616254519</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.934941983401482</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-5.815837257575128</v>
+        <v>-5.815837257434911</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.23577657025787</v>
+        <v>46.23577715539861</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>9.103864503199361</v>
+        <v>9.103864649271475</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>1.560135065854949</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1214513132016611</v>
+        <v>-0.121451313682109</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.22630981911153</v>
+        <v>52.22630985095005</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>13.04338897257761</v>
+        <v>13.04338885363556</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4506725487651918</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.444089150789291</v>
+        <v>-0.4440891515321899</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>311.9804891749366</v>
+        <v>311.980489174938</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>50.5</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>38.12016304578459</v>
+        <v>38.12016311522286</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>6.852570144367955</v>
+        <v>6.852569993156149</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>2.427258755264709</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.02594204660493094</v>
+        <v>-0.02594204666099717</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>308.8541683362196</v>
+        <v>308.8541683362195</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>74.09999999999999</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>37.21330444108085</v>
+        <v>37.21330496129914</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>9.465805422527808</v>
+        <v>9.465805455445979</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.9879476334987756</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.2680275236563803</v>
+        <v>-0.2680275238526175</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>48.09318561686796</v>
+        <v>48.09318560519053</v>
       </c>
       <c r="I80" s="2" t="n">
         <v>15.26455533280837</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.06866616052791649</v>
+        <v>-0.06866616047183249</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>42.26263508135629</v>
+        <v>42.26263505807903</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>13.48209430188449</v>
+        <v>13.48209429719711</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.5314520845681304</v>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>282.251971329263</v>
+        <v>282.2519713292633</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>97.3</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>33.0066884658544</v>
+        <v>33.00668855393134</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>27.51638200017733</v>
+        <v>27.51638209591686</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.513697526763331</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.4252203472449203</v>
+        <v>-0.4252203476654333</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>39.636476738601</v>
+        <v>39.63647675281566</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>29.14200504635948</v>
+        <v>29.14200513778649</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.7055078030690214</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-1.92155247161646</v>
+        <v>-1.921552468532762</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>275.8955318291405</v>
+        <v>275.8955318291406</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>213</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>32.17204049819425</v>
+        <v>32.17204053151654</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>18.61855957768476</v>
+        <v>18.61855965765578</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.4418196652627401</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-4.277029717507125</v>
+        <v>-4.277029717675313</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>39.7425334334281</v>
+        <v>39.7425334415413</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>19.82601724467363</v>
+        <v>19.82601734464073</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.730924899218151</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-30.57943230678627</v>
+        <v>-30.57943231071072</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>38.50361059945103</v>
+        <v>38.50361063387068</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>16.77364683899512</v>
+        <v>16.77364686166716</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.6177546508757084</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.3803953205665522</v>
+        <v>-0.380395320818852</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>38.74714832246571</v>
+        <v>38.74714783330152</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>22.87808890839352</v>
+        <v>22.8780889848114</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.031704685850572</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.1915744321265964</v>
+        <v>-0.1915744322667622</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>257.774819400156</v>
+        <v>257.7748194001568</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>26</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>48.15529523425525</v>
+        <v>48.15529530021113</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>19.71079933393996</v>
+        <v>19.71079938292834</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>1.649037471566105</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.1667650628364989</v>
+        <v>-0.1667650629906861</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>256.7303568862035</v>
+        <v>256.7303568862033</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>27.9</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>37.16357542663297</v>
+        <v>37.16357538838862</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>16.87350930133317</v>
+        <v>16.87350925920635</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.6220159686264627</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.2109864397250648</v>
+        <v>-0.2109864397110513</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>40.77252145651015</v>
+        <v>40.77252154277039</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>21.96379936653261</v>
+        <v>21.96379932562726</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.4918371564372804</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.01557640348948058</v>
+        <v>-0.01557640353153306</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>44.55140987825153</v>
+        <v>44.55140991743646</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>13.96089788036257</v>
+        <v>13.96089770128274</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-1.425587248291268</v>
+        <v>-1.425587248627676</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>237.881670588738</v>
+        <v>237.8816705887381</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>127.5</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>34.9198795097312</v>
+        <v>34.91987954716525</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>12.97696206154622</v>
+        <v>12.97696210844495</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.8352331012409452</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.8782033290567237</v>
+        <v>-0.8782033297575751</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>234.2400448020724</v>
+        <v>234.2400448020728</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>89.2</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>35.12404480539568</v>
+        <v>35.12404516396292</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.93071944941106</v>
+        <v>17.93071957472839</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.9621708467024712</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.4948365706663271</v>
+        <v>-0.4948365745910894</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>232.5910084003217</v>
+        <v>232.5910084003216</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>72.5</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>39.68120863300165</v>
+        <v>39.68120857977471</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>13.54440825772829</v>
+        <v>13.54440836878628</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.8367183991488116</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.4773424468042709</v>
+        <v>-0.4773424464117937</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>42.40987572787235</v>
+        <v>42.40987573464388</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>18.66631845639528</v>
+        <v>18.66631862181538</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.2388615937016738</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.6066177946856586</v>
+        <v>-0.6066177946576288</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>36.33721909884041</v>
+        <v>36.33721911774246</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>11.89911400838402</v>
+        <v>11.89911408489632</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.7088647421102982</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.6654665395920856</v>
+        <v>-0.6654665395640569</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>41.04106353926579</v>
+        <v>41.04106365038107</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.5445837894609</v>
+        <v>14.54458377371955</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.5793334974259351</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-1.794214876882355</v>
+        <v>-1.794214879125021</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>220.8907140876718</v>
+        <v>220.8907140876705</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>48.2</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.72261151552643</v>
+        <v>42.7226114936282</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.44028203172052</v>
+        <v>19.44028202468623</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.6455369966166463</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.2127286604690019</v>
+        <v>-0.2127286604409696</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>40.68829056401932</v>
+        <v>40.68829057730525</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>19.30406058612635</v>
+        <v>19.30406054645067</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.3277851763556027</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-2.662322785978386</v>
+        <v>-2.662322786034475</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>215.1517507111491</v>
+        <v>215.1517507111496</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>4890</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>39.87430340127597</v>
+        <v>39.87430339762433</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>16.0726909347484</v>
+        <v>16.07269091214538</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.732448737896305</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-75.60938772808734</v>
+        <v>-75.60938772668523</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>213.9925782522706</v>
+        <v>213.9925782522711</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>35.45</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>36.64448647962521</v>
+        <v>36.64448615213342</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>16.00795407161245</v>
+        <v>16.00795425620245</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.5427307671178602</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.1323493481122316</v>
+        <v>-0.1323493478879627</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.7441248890414</v>
+        <v>41.74412493609269</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>16.10483790391011</v>
+        <v>16.10483794033801</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.4215792906941168</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.102112702959697</v>
+        <v>-0.102112703001747</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         <v>38.75829517534873</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.03675806765995</v>
+        <v>12.0367580421686</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.4552798044629044</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>40.18137515989376</v>
+        <v>40.18137544932964</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>21.93048348874958</v>
+        <v>21.93048346021575</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.02958028798918</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.05609540916784084</v>
+        <v>0.05609540874734253</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>171.8923795645468</v>
+        <v>171.8923795645469</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>23.2</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>37.01438772758838</v>
+        <v>37.01438775780172</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>18.16634082012416</v>
+        <v>18.16634120023194</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.173065588498997</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.1595868389223357</v>
+        <v>-0.1595868391185751</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>43.07968354876465</v>
+        <v>43.07968339761172</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.12535518403117</v>
+        <v>16.12535523466551</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.491893028793488</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>47.70825010650694</v>
+        <v>47.70825042663109</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>11.32705217296843</v>
+        <v>11.32705202112528</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.7033086634740966</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.06779734590866815</v>
+        <v>0.06779734564234507</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>151.7663236061505</v>
+        <v>151.7663236061507</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>1410</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>39.04530025725249</v>
+        <v>39.04530018387027</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>18.20537912989366</v>
+        <v>18.20537911898719</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.6093792743911375</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-25.85459688476932</v>
+        <v>-25.85459686850967</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>136.2855693354545</v>
+        <v>136.2855693354553</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>32.25</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>38.03114515793416</v>
+        <v>38.03114442274243</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.87114529187345</v>
+        <v>18.87114541205426</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.2637962126132823</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.2893208650783236</v>
+        <v>-0.2893208637887592</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>39.4292838588584</v>
+        <v>39.42928396553069</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>21.49564508367213</v>
+        <v>21.49564517636999</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.235452198499643</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.2875912624975255</v>
+        <v>-0.2875912625816328</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>41.00225265806684</v>
+        <v>41.00225269182219</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.92605770829745</v>
+        <v>18.92605770781575</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.501698398289172</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-2.423439907504846</v>
+        <v>-2.423439907967414</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>31.76191441561846</v>
+        <v>31.76191442993274</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>11.60455407689306</v>
+        <v>11.60455413410972</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>1.186004476211294</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.2726743077764512</v>
+        <v>-0.2726743078605591</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>106.2281384094414</v>
+        <v>106.2281384094417</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>18.5</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>49.17189695544685</v>
+        <v>49.17189696005254</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>6.537717299968499</v>
+        <v>6.537717339499033</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.762763858258577</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.02907943214468557</v>
+        <v>0.02907943210263628</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>57.88731979447366</v>
+        <v>57.88731979447398</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>72.3</v>
@@ -6488,7 +6488,7 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>35.16830381854814</v>
+        <v>35.16830362498676</v>
       </c>
       <c r="I114" s="2" t="n">
         <v>15.5730388209383</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.06504822850717429</v>
+        <v>0.06504822878750138</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>40.45289783597504</v>
+        <v>40.45289783597484</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>56.5</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>22.82307701330924</v>
+        <v>22.82307732613796</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>16.14584114068564</v>
+        <v>16.14584101148633</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.6973022282200585</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.2827038231396533</v>
+        <v>-0.282703823307857</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>21.31005534658615</v>
+        <v>21.31005534658614</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>17.95</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>48.51248972795864</v>
+        <v>48.51248975829579</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>9.310229865554501</v>
+        <v>9.310229858511908</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.1556555978811549</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0881060235645888</v>
+        <v>0.08810602338236645</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>

</xml_diff>